<commit_message>
Tighten sugar news summaries
</commit_message>
<xml_diff>
--- a/reports/2026/08/Sugar News 2026-08-05.xlsx
+++ b/reports/2026/08/Sugar News 2026-08-05.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -513,63 +513,63 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>印度政府披露糖厂运行和压榨安排，数据为17%。糖厂运行变化会直接影响甘蔗入榨、压榨节奏和阶段性食糖产量。来源：The Economic Times（https://news.google.com/rss/articles/CBMi3wFBVV95cUxOdElYdGNjM0phLUNJbHZTZXpCUEtsLTE3SDd0aDU2SDhPWDh0Zzl2SzRfcUFrNXN1Q19IV1hJdFdpbS1BTmRzVC1RNjF0YTItVmZvQ2kzYkk0RmFHa1pJNFFYYlRTSEhNSUJ6RGE5UDcxeEIzQ3FXcmhBTFNsa3A5WDY1Uk5WYkRST2JiYzhSWWV6dDZOQm1lOWN6aWRPZXBKUnRqNXRuS2pKWjRPdWd4SGpYMzJRLVdOdWplUTkxU1BnbFcyYlNZMFpIb19FSzhkSlM2UmF5UUF1WVRSV1lr0gHkAUFVX3lxTE1MZzd1MDlLMDAxaWZQbkNNRG5FZVJxNjFldFo1MHVYWGpQMHZIdFpXV2pVQjRGNXFWeWNVREtUZk9vREdBcVZxNzBLb0VWTDRRS1FTcFlqeDd0dElCNkJLeUE3MS1sRG9naE1BeVRETjBzZEY5cW5za2taRzJGMzA4ZjBfSV90UkRMZFgyMnZyYUlfLW5RVml3M0FLcEttMk5WWWZwaTZLTGtHcEpIUzBMVFQtVEtZUXhpV01pSmlqdTFETUsybnhDRnNjN0U0Yzg5VGlZWl9JOTBlTmdoWm11bkhUeQ?oc=5）</t>
+          <t>印度糖价一个月上涨17%，糖厂预计政府会在库存限制落地后继续加强市场调控。库存限制压缩贸易商和终端囤货空间，削弱价格上涨后的补库需求，短期利空印度现货糖价。来源：The Economic Times（https://news.google.com/rss/articles/CBMi3wFBVV95cUxOdElYdGNjM0phLUNJbHZTZXpCUEtsLTE3SDd0aDU2SDhPWDh0Zzl2SzRfcUFrNXN1Q19IV1hJdFdpbS1BTmRzVC1RNjF0YTItVmZvQ2kzYkk0RmFHa1pJNFFYYlRTSEhNSUJ6RGE5UDcxeEIzQ3FXcmhBTFNsa3A5WDY1Uk5WYkRST2JiYzhSWWV6dDZOQm1lOWN6aWRPZXBKUnRqNXRuS2pKWjRPdWd4SGpYMzJRLVdOdWplUTkxU1BnbFcyYlNZMFpIb19FSzhkSlM2UmF5UUF1WVRSV1lr0gHkAUFVX3lxTE1MZzd1MDlLMDAxaWZQbkNNRG5FZVJxNjFldFo1MHVYWGpQMHZIdFpXV2pVQjRGNXFWeWNVREtUZk9vREdBcVZxNzBLb0VWTDRRS1FTcFlqeDd0dElCNkJLeUE3MS1sRG9naE1BeVRETjBzZEY5cW5za2taRzJGMzA4ZjBfSV90UkRMZFgyMnZyYUlfLW5RVml3M0FLcEttMk5WWWZwaTZLTGtHcEpIUzBMVFQtVEtZUXhpV01pSmlqdTFETUsybnhDRnNjN0U0Yzg5VGlZWl9JOTBlTmdoWm11bkhUeQ?oc=5）</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>利空：糖厂运行、压榨能力或原料供应改善会提高食糖生产节奏，增加阶段性供应。</t>
+          <t>利空：库存限制会压缩贸易商和终端囤货空间，削弱价格上涨后的补库需求，短期压制印度现货糖价。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="180" customHeight="1" s="2">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>泰国</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>印度糖业市场发布或调整食糖价格和市场流通，数据为17%。报价变化会反映现货供需松紧和贸易商补库意愿。来源：Whalesbook（https://news.google.com/rss/articles/CBMi1gFBVV95cUxPQ0ZCdGNveDFJaGlIcGVlY3BwU3drY1hCeWUzdnFtd0ZrZ3hmaUdVZ3N0Y0dmQk1mSjhsTVVhLXFpY191VWJLa1FNSTRIMzkzSGpETzNXaUdDMVI4UFo1UldNSFFYTVA1MDJwTE5aTTR2REVidnFLc0NaZV85LWxMSDBhQ1JXRWRuaWE1emtDallTalNyV0pKbzhEd0NwOFg5eUFWcEtoQ2JvTFpyQTJ2SkdlTE01cllqWTB2S0w5T0pTcHhCSFpRWVRveTFqNUJtdm40a1dB?oc=5）</t>
+          <t>Open-Meteo预报显示（2026-08-06至2026-08-12），泰国东北部（呵叻、孔敬、乌隆他尼、猜也蓬）；北部（那空沙旺、甘烹碧、素可泰、彭世洛）；中部及西部（北碧、华富里、素攀武里、猜纳）；东部（沙缴、春武里）等主要甘蔗产区存在降雨预报，实际可用预报期为7日，累计预测降雨较高的监测点包括素可泰约132.7mm、甘烹碧约131.9mm、乌隆他尼约120.4mm。当前处于甘蔗生长阶段，降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：Open-Meteo（https://api.open-meteo.com/v1/forecast）</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>中性：价格信息缺少明确涨跌幅或区域基准，暂不改变供需判断。</t>
+          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="180" customHeight="1" s="2">
+    <row r="4" ht="118.05" customHeight="1" s="2">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>泰国</t>
+          <t>中国</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Open-Meteo预报显示（2026-08-06至2026-08-12），泰国东北部（呵叻、孔敬、乌隆他尼、猜也蓬）；北部（那空沙旺、甘烹碧、素可泰、彭世洛）；中部及西部（北碧、华富里、素攀武里、猜纳）；东部（沙缴、春武里）等主要甘蔗产区存在降雨预报，实际可用预报期为7日，累计预测降雨较高的监测点包括素可泰约132.7mm、甘烹碧约131.9mm、乌隆他尼约120.4mm。当前处于甘蔗生长阶段，降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：Open-Meteo（https://api.open-meteo.com/v1/forecast）</t>
+          <t>已完成中国食糖、甘蔗、甜菜糖、进口、库存、现货价格和主产区天气等重点方向监测，未发现符合收录标准的新增重要糖业事件。该结果仅表示本次公开来源检索没有可发布的新事件，不代表中国食糖供需或价格没有变化。来源：Sugar News中国糖业每日监测日志（https://github.com/lishi2626/sugar-news/actions）</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
+          <t>中性：本次监测未发现足以改变中国食糖供需、库存、进口或价格预期的新增公开信息。</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="118.05" customHeight="1" s="2">
+    <row r="5" ht="180" customHeight="1" s="2">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>中国</t>
+          <t>菲律宾</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>已完成中国食糖、甘蔗、甜菜糖、进口、库存、现货价格和主产区天气等重点方向监测，未发现符合收录标准的新增重要糖业事件。该结果仅表示本次公开来源检索没有可发布的新事件，不代表中国食糖供需或价格没有变化。来源：Sugar News中国糖业每日监测日志（https://github.com/lishi2626/sugar-news/actions）</t>
+          <t>菲律宾东内格罗斯省因甘蔗虫害扩散寻求国家援助，地方政府希望中央支持受灾蔗农和防控行动。虫害扩散会压低受害地块单产并增加蔗农补救成本，若防控资金不到位，内格罗斯糖料供应稳定性下降，利多糖价。来源：Daily Guardian（https://news.google.com/rss/articles/CBMimgFBVV95cUxQOGlwVzdSS1J3bV9FUjBwdnpVTHJFaHNHeFlmM1BHeGpuTFdQazB6UjhRV3pzY0dlVW5kTFMyd2tCdWREQXRkZEFqTElaOUhaM3VzUnZ4X1ctNjJOWDlsYUNwczZYakQ2MXhSWXVObHlWb1lQMVR4a3dzVVBkdjJqOS1nMnJvRU9wMGcyNnJ3TGlBYjlHY2xTdVR3?oc=5）</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>中性：本次监测未发现足以改变中国食糖供需、库存、进口或价格预期的新增公开信息。</t>
+          <t>利多：东内格罗斯甘蔗虫害扩散并需要国家援助，说明地方防控和蔗农现金流压力上升，若处置不及时将削弱糖料供应稳定性。</t>
         </is>
       </c>
     </row>
@@ -581,29 +581,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>菲律宾主产区农业或气象机构预警甘蔗产区天气、干旱或病虫害，具体幅度未披露。产区天气或病虫害变化会影响甘蔗生长、收割和糖料供应稳定性。来源：Daily Guardian（https://news.google.com/rss/articles/CBMimgFBVV95cUxQOGlwVzdSS1J3bV9FUjBwdnpVTHJFaHNHeFlmM1BHeGpuTFdQazB6UjhRV3pzY0dlVW5kTFMyd2tCdWREQXRkZEFqTElaOUhaM3VzUnZ4X1ctNjJOWDlsYUNwczZYakQ2MXhSWXVObHlWb1lQMVR4a3dzVVBkdjJqOS1nMnJvRU9wMGcyNnJ3TGlBYjlHY2xTdVR3?oc=5）</t>
+          <t>菲律宾西内格罗斯省虫害防控工作组已用真菌处理77.3公顷甘蔗虫害地块，并计划把防治推进到另外3个地方政府辖区。生物防治扩大有助于压低虫害继续蔓延的风险，但已处理面积说明内格罗斯蔗区仍存在虫害压力，短期利多糖价。来源：Digicast Negros（https://news.google.com/rss/articles/CBMi0AFBVV95cUxQOTZENTdONWVQMG5kVnB4OXc0RWltWkNRb1cxZWRZRW5qRDBic1dEcExQRFlIWDRZbThiMGZ0SUtoalpZWW1RNWNUWGNBU1ZNYVV1MkFyZEROeHBFVzVoRWVranlHcHBQaUczSTZ4Q1locXRLQldVM0xTa01oU0FnYUZBaVZsMWx3VlhUckZteUdxaEJhb2dkTlVaaE9tOUJhOUJldkUyOFY1QVZCRUlSUldpZlFhQ1JDcTQybFlZS014dkJHbXhJbkVuWjJ6alAt0gHWAUFVX3lxTE5ya1Y1cFcxTDhlZU9IRWlPelZTdWVLZnVrbHEtcU8tZVMwbVRuTk0tSUlzaXVYRkpvbkxqSTlnck1VeGEtODJLT1YyTWttdGZteXBXREEwcFZ2eHRES29XcDZqR3c3Uk5UZTZPVkloR01MVHNjUElpQzMxX0xvczE3cEUwZGhNQkQ2ckNSSnFzaThFZzhBbnVJY1M2bXhsVWV5UjEzOW5ycGphZ0w0S2tmZ1R3TTZsT0d6a0FuSUNud3JFRklCWHM0WDB1UElCSkx5c2kxa0E?oc=5）</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>利多：干旱、洪涝或病虫害会压低甘蔗单产并削弱糖料供应稳定性，从而支撑糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="180" customHeight="1" s="2">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>菲律宾</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>菲律宾主产区农业或气象机构预警甘蔗产区天气、干旱或病虫害，数据为77.3公顷。产区天气或病虫害变化会影响甘蔗生长、收割和糖料供应稳定性。来源：Digicast Negros（https://news.google.com/rss/articles/CBMi0AFBVV95cUxQOTZENTdONWVQMG5kVnB4OXc0RWltWkNRb1cxZWRZRW5qRDBic1dEcExQRFlIWDRZbThiMGZ0SUtoalpZWW1RNWNUWGNBU1ZNYVV1MkFyZEROeHBFVzVoRWVranlHcHBQaUczSTZ4Q1locXRLQldVM0xTa01oU0FnYUZBaVZsMWx3VlhUckZteUdxaEJhb2dkTlVaaE9tOUJhOUJldkUyOFY1QVZCRUlSUldpZlFhQ1JDcTQybFlZS014dkJHbXhJbkVuWjJ6alAt0gHWAUFVX3lxTE5ya1Y1cFcxTDhlZU9IRWlPelZTdWVLZnVrbHEtcU8tZVMwbVRuTk0tSUlzaXVYRkpvbkxqSTlnck1VeGEtODJLT1YyTWttdGZteXBXREEwcFZ2eHRES29XcDZqR3c3Uk5UZTZPVkloR01MVHNjUElpQzMxX0xvczE3cEUwZGhNQkQ2ckNSSnFzaThFZzhBbnVJY1M2bXhsVWV5UjEzOW5ycGphZ0w0S2tmZ1R3TTZsT0d6a0FuSUNud3JFRklCWHM0WDB1UElCSkx5c2kxa0E?oc=5）</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>利多：干旱、洪涝或病虫害会压低甘蔗单产并削弱糖料供应稳定性，从而支撑糖价。</t>
+          <t>利多：西内格罗斯已出现需要集中处理的甘蔗虫害地块，若真菌防治未能及时控制扩散，将压低受害区域单产并削弱糖料供应稳定性。</t>
         </is>
       </c>
     </row>

</xml_diff>